<commit_message>
Cambios estructurales en seleccion de pacientes y denominacion archivos
</commit_message>
<xml_diff>
--- a/Output/Tables/Table_2_by_org_inicial.xlsx
+++ b/Output/Tables/Table_2_by_org_inicial.xlsx
@@ -340,7 +340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -351,27 +351,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>[ALL]   N=2166</t>
+          <t>[ALL]   N=1949</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Equip_Atdom   N=777</t>
+          <t>Equip_Atdom   N=708</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Equip_Inf   N=308</t>
+          <t>Equip_Inf   N=278</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>UAB_consulta   N=384</t>
+          <t>UAB_consulta   N=339</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>UAB_consulta_reforc   N=697</t>
+          <t>UAB_consulta_reforc   N=624</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -383,180 +383,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sex (female), N (%):</t>
+          <t>Sex (female), N (%)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  1396 (71.6%)  </t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  506 (71.5%)   </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  216 (77.7%)   </t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  224 (66.1%)   </t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    450 (72.1%)    </t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.034  </t>
+          <t xml:space="preserve">  0.016  </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    No</t>
+          <t>Age (years), Median [25th;75th]</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  599 (27.7%)   </t>
+          <t>90.7 [85.8;94.6]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  222 (28.6%)   </t>
+          <t>89.8 [84.6;94.0]</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   67 (21.8%)   </t>
+          <t>92.2 [87.4;96.0]</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  125 (32.6%)   </t>
+          <t>90.9 [86.1;94.8]</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">    185 (26.5%)    </t>
+          <t xml:space="preserve"> 91.1 [86.6;94.7]  </t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Yes</t>
+          <t>Years in home-based program, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1566 (72.3%)  </t>
+          <t>2.12 [1.18;3.96]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  555 (71.4%)   </t>
+          <t>2.23 [1.25;4.09]</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  241 (78.2%)   </t>
+          <t>2.54 [1.25;4.06]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  259 (67.4%)   </t>
+          <t>1.86 [1.13;3.19]</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">    511 (73.3%)    </t>
+          <t xml:space="preserve"> 1.93 [1.14;3.93]  </t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve">  0.006  </t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t>High comorbidity status (AMG index ≥p85), N (%)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1 (0.05%)    </t>
+          <t xml:space="preserve">  1838 (94.3%)  </t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">  678 (95.8%)   </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">  263 (94.6%)   </t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">  319 (94.1%)   </t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">     1 (0.14%)     </t>
+          <t xml:space="preserve">    578 (92.6%)    </t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve">  0.105  </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Age (years), Median [25th;75th]</t>
+          <t>No. registered chronic diseases, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>90.8 [86.0;94.6]</t>
+          <t>11.0 [8.00;14.0]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>89.8 [84.6;93.8]</t>
+          <t>12.0 [9.00;15.0]</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>92.3 [87.4;96.1]</t>
+          <t>11.0 [9.00;14.8]</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>90.7 [85.7;94.8]</t>
+          <t>11.0 [8.00;14.0]</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 91.1 [86.8;94.6]  </t>
+          <t xml:space="preserve"> 10.0 [7.00;14.0]  </t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -568,106 +568,106 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Years in home-based program, Median [25th;75th]</t>
+          <t>Commorbidity and complexity, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2.14 [1.18;3.96]</t>
+          <t>18.6 [13.6;24.5]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.21 [1.22;4.05]</t>
+          <t>20.1 [15.0;25.8]</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.54 [1.24;4.18]</t>
+          <t>18.2 [13.2;23.6]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.86 [1.12;3.39]</t>
+          <t>18.5 [13.8;23.2]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2.03 [1.16;3.96]  </t>
+          <t xml:space="preserve"> 17.4 [12.3;23.5]  </t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.013  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>High comorbidity status (AMG index ≥p85), N (%)</t>
+          <t>Fragil Vig index, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2042 (94.3%)  </t>
+          <t>0.36 [0.28;0.48]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  747 (96.1%)   </t>
+          <t>0.36 [0.28;0.44]</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  289 (93.8%)   </t>
+          <t>0.36 [0.24;0.48]</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  359 (93.5%)   </t>
+          <t>0.36 [0.24;0.52]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    647 (92.8%)    </t>
+          <t xml:space="preserve"> 0.40 [0.28;0.48]  </t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.041  </t>
+          <t xml:space="preserve">  0.491  </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>No. registered chronic diseases, Median [25th;75th]</t>
+          <t>PCC, N (%)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>11.0 [8.00;14.0]</t>
+          <t xml:space="preserve">  1526 (78.3%)  </t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12.0 [9.00;15.0]</t>
+          <t xml:space="preserve">  591 (83.5%)   </t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11.0 [9.00;14.0]</t>
+          <t xml:space="preserve">  151 (54.3%)   </t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11.0 [8.00;14.0]</t>
+          <t xml:space="preserve">  274 (80.8%)   </t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10.0 [8.00;14.0]  </t>
+          <t xml:space="preserve">    510 (81.7%)    </t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -679,217 +679,217 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Commorbidity and complexity, Median [25th;75th]</t>
+          <t>MACA, N (%)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.6 [13.7;24.4]</t>
+          <t xml:space="preserve">  160 (8.21%)   </t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>20.1 [15.1;25.7]</t>
+          <t xml:space="preserve">   63 (8.90%)   </t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>18.2 [13.3;23.5]</t>
+          <t xml:space="preserve">   31 (11.2%)   </t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>18.2 [13.7;23.0]</t>
+          <t xml:space="preserve">   27 (7.96%)   </t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17.6 [12.4;23.4]  </t>
+          <t xml:space="preserve">    39 (6.25%)     </t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.077  </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Fragil Vig index, Median [25th;75th]</t>
+          <t>Dependency according to Barthel Index for Activities of Daily Living, N (%):</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.36 [0.28;0.48]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.36 [0.28;0.44]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.34 [0.25;0.44]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0.40 [0.28;0.48]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.36 [0.28;0.48]  </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.429  </t>
+          <t xml:space="preserve">  0.008  </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PCC, N (%)</t>
+          <t xml:space="preserve">    Total (&lt;20)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1706 (78.8%)  </t>
+          <t xml:space="preserve">  208 (10.7%)   </t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  653 (84.0%)   </t>
+          <t xml:space="preserve">   67 (9.46%)   </t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  171 (55.5%)   </t>
+          <t xml:space="preserve">   28 (10.1%)   </t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  312 (81.2%)   </t>
+          <t xml:space="preserve">   38 (11.2%)   </t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    570 (81.8%)    </t>
+          <t xml:space="preserve">    75 (12.0%)     </t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MACA, N (%)</t>
+          <t xml:space="preserve">    Severe (20-35)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  171 (7.89%)   </t>
+          <t xml:space="preserve">  256 (13.1%)   </t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   65 (8.37%)   </t>
+          <t xml:space="preserve">   84 (11.9%)   </t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   33 (10.7%)   </t>
+          <t xml:space="preserve">   41 (14.7%)   </t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   29 (7.55%)   </t>
+          <t xml:space="preserve">   45 (13.3%)   </t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    44 (6.31%)     </t>
+          <t xml:space="preserve">    86 (13.8%)     </t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.108  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dependency according to Barthel Index for Activities of Daily Living, N (%):</t>
+          <t xml:space="preserve">    Moderate (40-55)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  453 (23.2%)   </t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  140 (19.8%)   </t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   72 (25.9%)   </t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   71 (20.9%)   </t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    170 (27.2%)    </t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Total (&lt;20)</t>
+          <t xml:space="preserve">    Low (60-99)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  228 (10.5%)   </t>
+          <t xml:space="preserve">  991 (50.8%)   </t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   70 (9.01%)   </t>
+          <t xml:space="preserve">  407 (57.5%)   </t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   30 (9.74%)   </t>
+          <t xml:space="preserve">  130 (46.8%)   </t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   47 (12.2%)   </t>
+          <t xml:space="preserve">  175 (51.6%)   </t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    81 (11.6%)     </t>
+          <t xml:space="preserve">    279 (44.7%)    </t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -901,32 +901,32 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Severe (20-35)</t>
+          <t xml:space="preserve">    None (100)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  274 (12.7%)   </t>
+          <t xml:space="preserve">   33 (1.69%)   </t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   91 (11.7%)   </t>
+          <t xml:space="preserve">   8 (1.13%)    </t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   43 (14.0%)   </t>
+          <t xml:space="preserve">   5 (1.80%)    </t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   49 (12.8%)   </t>
+          <t xml:space="preserve">   7 (2.06%)    </t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">    91 (13.1%)     </t>
+          <t xml:space="preserve">    13 (2.08%)     </t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -938,32 +938,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Moderate (40-55)</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  506 (23.4%)   </t>
+          <t xml:space="preserve">   8 (0.41%)    </t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  150 (19.3%)   </t>
+          <t xml:space="preserve">   2 (0.28%)    </t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   83 (26.9%)   </t>
+          <t xml:space="preserve">   2 (0.72%)    </t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   84 (21.9%)   </t>
+          <t xml:space="preserve">   3 (0.88%)    </t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">    189 (27.1%)    </t>
+          <t xml:space="preserve">     1 (0.16%)     </t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -975,69 +975,69 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Low (60-99)</t>
+          <t>Short Portable Mental Status Questionnaire, N (%):</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1107 (51.1%)  </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  455 (58.6%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  144 (46.8%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  193 (50.3%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    315 (45.2%)    </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve">  0.201  </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    None (100)</t>
+          <t xml:space="preserve">    No deficit (0-2 mistakes)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   41 (1.89%)   </t>
+          <t xml:space="preserve">  1060 (54.4%)  </t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (1.03%)    </t>
+          <t xml:space="preserve">  387 (54.7%)   </t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   6 (1.95%)    </t>
+          <t xml:space="preserve">  147 (52.9%)   </t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (2.08%)    </t>
+          <t xml:space="preserve">  191 (56.3%)   </t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    19 (2.73%)     </t>
+          <t xml:space="preserve">    335 (53.7%)    </t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1049,32 +1049,32 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    Low (3-4 mistakes)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   10 (0.46%)   </t>
+          <t xml:space="preserve">  288 (14.8%)   </t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.39%)    </t>
+          <t xml:space="preserve">  110 (15.5%)   </t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2 (0.65%)    </t>
+          <t xml:space="preserve">   39 (14.0%)   </t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.78%)    </t>
+          <t xml:space="preserve">   48 (14.2%)   </t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">     2 (0.29%)     </t>
+          <t xml:space="preserve">    91 (14.6%)     </t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1086,69 +1086,69 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Short Portable Mental Status Questionnaire, N (%):</t>
+          <t xml:space="preserve">    Moderate (5-7 mistakes)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  266 (13.6%)   </t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   79 (11.2%)   </t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   42 (15.1%)   </t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   47 (13.9%)   </t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    98 (15.7%)     </t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.436  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    No deficit (0-2 mistakes)</t>
+          <t xml:space="preserve">    Severe (8-10 mistakes)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1161 (53.6%)  </t>
+          <t xml:space="preserve">  322 (16.5%)   </t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  418 (53.8%)   </t>
+          <t xml:space="preserve">  129 (18.2%)   </t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  166 (53.9%)   </t>
+          <t xml:space="preserve">   45 (16.2%)   </t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  208 (54.2%)   </t>
+          <t xml:space="preserve">   50 (14.7%)   </t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    369 (52.9%)    </t>
+          <t xml:space="preserve">    98 (15.7%)     </t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1160,32 +1160,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Low (3-4 mistakes)</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  327 (15.1%)   </t>
+          <t xml:space="preserve">   13 (0.67%)   </t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  124 (16.0%)   </t>
+          <t xml:space="preserve">   3 (0.42%)    </t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">   46 (14.9%)   </t>
+          <t xml:space="preserve">   5 (1.80%)    </t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">   55 (14.3%)   </t>
+          <t xml:space="preserve">   3 (0.88%)    </t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    102 (14.6%)    </t>
+          <t xml:space="preserve">     2 (0.32%)     </t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1197,69 +1197,69 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Moderate (5-7 mistakes)</t>
+          <t>Incontinence, N (%):</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  300 (13.9%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   89 (11.5%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   44 (14.3%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   59 (15.4%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    108 (15.5%)    </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve">  0.059  </t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Severe (8-10 mistakes)</t>
+          <t xml:space="preserve">    Fecal and urinary</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  362 (16.7%)   </t>
+          <t xml:space="preserve">  248 (12.7%)   </t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  142 (18.3%)   </t>
+          <t xml:space="preserve">   91 (12.9%)   </t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   47 (15.3%)   </t>
+          <t xml:space="preserve">   44 (15.8%)   </t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   59 (15.4%)   </t>
+          <t xml:space="preserve">   46 (13.6%)   </t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    114 (16.4%)    </t>
+          <t xml:space="preserve">    67 (10.7%)     </t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1271,32 +1271,32 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    Fecal</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   16 (0.74%)   </t>
+          <t xml:space="preserve">   8 (0.41%)    </t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   4 (0.51%)    </t>
+          <t xml:space="preserve">   5 (0.71%)    </t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   5 (1.62%)    </t>
+          <t xml:space="preserve">   2 (0.72%)    </t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.78%)    </t>
+          <t xml:space="preserve">   1 (0.29%)    </t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">     4 (0.57%)     </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1308,69 +1308,69 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Incontinence, N (%):</t>
+          <t xml:space="preserve">    Urinary</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  1002 (51.4%)  </t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  374 (52.8%)   </t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  150 (54.0%)   </t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  165 (48.7%)   </t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    313 (50.2%)    </t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  0.020  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Fecal and urinary</t>
+          <t xml:space="preserve">    None/None registered</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  265 (12.2%)   </t>
+          <t xml:space="preserve">  691 (35.5%)   </t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   92 (11.8%)   </t>
+          <t xml:space="preserve">  238 (33.6%)   </t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   46 (14.9%)   </t>
+          <t xml:space="preserve">   82 (29.5%)   </t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   55 (14.3%)   </t>
+          <t xml:space="preserve">  127 (37.5%)   </t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">    72 (10.3%)     </t>
+          <t xml:space="preserve">    244 (39.1%)    </t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1382,69 +1382,69 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Fecal</t>
+          <t>Social risk, N (%):</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (0.37%)    </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   5 (0.64%)    </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2 (0.65%)    </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1 (0.26%)    </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Urinary</t>
+          <t xml:space="preserve">    No</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1122 (51.8%)  </t>
+          <t xml:space="preserve">  1165 (59.8%)  </t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  420 (54.1%)   </t>
+          <t xml:space="preserve">  558 (78.8%)   </t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  167 (54.2%)   </t>
+          <t xml:space="preserve">  177 (63.7%)   </t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  184 (47.9%)   </t>
+          <t xml:space="preserve">  149 (44.0%)   </t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">    351 (50.4%)    </t>
+          <t xml:space="preserve">    281 (45.0%)    </t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1456,32 +1456,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">    None/None registered</t>
+          <t xml:space="preserve">    Yes</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  771 (35.6%)   </t>
+          <t xml:space="preserve">  231 (11.9%)   </t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  260 (33.5%)   </t>
+          <t xml:space="preserve">   71 (10.0%)   </t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">   93 (30.2%)   </t>
+          <t xml:space="preserve">   93 (33.5%)   </t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">  144 (37.5%)   </t>
+          <t xml:space="preserve">   18 (5.31%)   </t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">    274 (39.3%)    </t>
+          <t xml:space="preserve">    49 (7.85%)     </t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1493,405 +1493,294 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Social risk, N (%):</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  553 (28.4%)   </t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   79 (11.2%)   </t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   8 (2.88%)    </t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  172 (50.7%)   </t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    294 (47.1%)    </t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    No</t>
+          <t>Social Risk (TIRS numeric), Median [25th;75th]</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1293 (59.7%)  </t>
+          <t>0.00 [0.00;1.00]</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  611 (78.6%)   </t>
+          <t>0.00 [0.00;1.00]</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  193 (62.7%)   </t>
+          <t>0.00 [0.00;1.00]</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  169 (44.0%)   </t>
+          <t>0.00 [0.00;1.00]</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    320 (45.9%)    </t>
+          <t xml:space="preserve"> 0.00 [0.00;1.00]  </t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Yes</t>
+          <t>Living alone, N (%)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  263 (12.1%)   </t>
+          <t xml:space="preserve">  383 (19.7%)   </t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   83 (10.7%)   </t>
+          <t xml:space="preserve">  182 (25.7%)   </t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  106 (34.4%)   </t>
+          <t xml:space="preserve">   59 (21.2%)   </t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   21 (5.47%)   </t>
+          <t xml:space="preserve">   38 (11.2%)   </t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">    53 (7.60%)     </t>
+          <t xml:space="preserve">    104 (16.7%)    </t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t>Need for any household adaptation, N (%)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  610 (28.2%)   </t>
+          <t xml:space="preserve">  510 (26.2%)   </t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   83 (10.7%)   </t>
+          <t xml:space="preserve">  246 (34.7%)   </t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   9 (2.92%)    </t>
+          <t xml:space="preserve">   66 (23.7%)   </t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  194 (50.5%)   </t>
+          <t xml:space="preserve">   68 (20.1%)   </t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    324 (46.5%)    </t>
+          <t xml:space="preserve">    130 (20.8%)    </t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Social Risk (TIRS numeric), Median [25th;75th]</t>
+          <t>Healthcare center, N (%):</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.00 [0.00;1.00]  </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.000  </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Living alone, N (%)</t>
+          <t xml:space="preserve">    Equip_Atdom</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  435 (20.1%)   </t>
+          <t xml:space="preserve">  708 (36.3%)   </t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  205 (26.4%)   </t>
+          <t xml:space="preserve">   708 (100%)   </t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   66 (21.4%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   48 (12.5%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    116 (16.6%)    </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Need for any household adaptation, N (%)</t>
+          <t xml:space="preserve">    Equip_Inf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  572 (26.4%)   </t>
+          <t xml:space="preserve">  278 (14.3%)   </t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  279 (35.9%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">   77 (25.0%)   </t>
+          <t xml:space="preserve">   278 (100%)   </t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">   78 (20.3%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    138 (19.8%)    </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Healthcare center, N (%):</t>
+          <t xml:space="preserve">    UAB_consulta</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  963 (49.4%)   </t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   339 (100%)   </t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
+          <t xml:space="preserve">    624 (100%)     </t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.000  </t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Equip_Atdom</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  777 (35.9%)   </t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   777 (100%)   </t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Equip_Inf</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  308 (14.2%)   </t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   308 (100%)   </t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    UAB_consulta</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1081 (49.9%)  </t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   384 (100%)   </t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    697 (100%)     </t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>

</xml_diff>

<commit_message>
Direcciones finales!!! ahora si n=2225
</commit_message>
<xml_diff>
--- a/Output/Tables/Table_2_by_org_inicial.xlsx
+++ b/Output/Tables/Table_2_by_org_inicial.xlsx
@@ -340,7 +340,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -351,30 +351,25 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>[ALL]   N=1949</t>
+          <t>Equip_Atdom   N=781</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Equip_Atdom   N=708</t>
+          <t>Equip_Inf   N=312</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Equip_Inf   N=278</t>
+          <t>UAB_consulta   N=411</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>UAB_consulta   N=339</t>
+          <t>UAB_consulta_reforc   N=720</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>UAB_consulta_reforc   N=624</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>p.overall</t>
         </is>
@@ -383,183 +378,158 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sex (female), N (%)</t>
+          <t>Sex (female), N (%):</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1396 (71.6%)  </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  506 (71.5%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  216 (77.7%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  224 (66.1%)   </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">    450 (72.1%)    </t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.016  </t>
+          <t xml:space="preserve">  0.109  </t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Age (years), Median [25th;75th]</t>
+          <t xml:space="preserve">    No</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>90.7 [85.8;94.6]</t>
+          <t xml:space="preserve">  196 (25.1%)   </t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>89.8 [84.6;94.0]</t>
+          <t xml:space="preserve">   63 (20.2%)   </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>92.2 [87.4;96.0]</t>
+          <t xml:space="preserve">  122 (29.7%)   </t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>90.9 [86.1;94.8]</t>
+          <t xml:space="preserve">    176 (24.4%)    </t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 91.1 [86.6;94.7]  </t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Years in home-based program, Median [25th;75th]</t>
+          <t xml:space="preserve">    Yes</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2.12 [1.18;3.96]</t>
+          <t xml:space="preserve">  481 (61.6%)   </t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.23 [1.25;4.09]</t>
+          <t xml:space="preserve">  205 (65.7%)   </t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.54 [1.25;4.06]</t>
+          <t xml:space="preserve">  232 (56.4%)   </t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.86 [1.13;3.19]</t>
+          <t xml:space="preserve">    456 (63.3%)    </t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1.93 [1.14;3.93]  </t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.006  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Distance from center (meters), Median [25th;75th]</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 761 [525;1067] </t>
+          <t xml:space="preserve">  104 (13.3%)   </t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 775 [572;1079] </t>
+          <t xml:space="preserve">   44 (14.1%)   </t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 481 [352;627]  </t>
+          <t xml:space="preserve">   57 (13.9%)   </t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1069 [815;1374] </t>
+          <t xml:space="preserve">    88 (12.2%)     </t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  748 [527;1036]   </t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Time_walking to center (minutes), Median [25th;75th]</t>
+          <t>Age (years), Median [25th;75th]</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>9.00 [6.00;13.0]</t>
+          <t>89.4 [84.1;93.7]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>9.00 [7.00;13.0]</t>
+          <t>91.3 [86.8;95.9]</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.00 [4.00;7.75]</t>
+          <t>90.6 [84.6;94.3]</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13.0 [10.0;16.5]</t>
+          <t xml:space="preserve"> 90.9 [85.4;94.4]  </t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 9.00 [6.00;12.0]  </t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
         <is>
           <t xml:space="preserve"> &lt;0.001  </t>
         </is>
@@ -568,109 +538,94 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>High comorbidity status (AMG index ≥p85), N (%)</t>
+          <t>Years in home-based program, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1838 (94.3%)  </t>
+          <t>2.04 [0.89;3.90]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  678 (95.8%)   </t>
+          <t>1.97 [0.84;3.67]</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  263 (94.6%)   </t>
+          <t>1.68 [0.82;3.14]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  319 (94.1%)   </t>
+          <t xml:space="preserve"> 1.82 [0.92;3.78]  </t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    578 (92.6%)    </t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.105  </t>
+          <t xml:space="preserve">  0.251  </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>No. registered chronic diseases, Median [25th;75th]</t>
+          <t>High comorbidity status (AMG index ≥p85), N (%)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>11.0 [8.00;14.0]</t>
+          <t xml:space="preserve">  750 (96.0%)   </t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12.0 [9.00;15.0]</t>
+          <t xml:space="preserve">  292 (93.6%)   </t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>11.0 [9.00;14.8]</t>
+          <t xml:space="preserve">  380 (92.5%)   </t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>11.0 [8.00;14.0]</t>
+          <t xml:space="preserve">    660 (91.7%)    </t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10.0 [7.00;14.0]  </t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.004  </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Commorbidity and complexity, Median [25th;75th]</t>
+          <t>No. registered chronic diseases, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>18.6 [13.6;24.5]</t>
+          <t>12.0 [9.00;15.0]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>20.1 [15.0;25.8]</t>
+          <t>11.0 [9.00;14.0]</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>18.2 [13.2;23.6]</t>
+          <t>11.0 [8.00;14.0]</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>18.5 [13.8;23.2]</t>
+          <t xml:space="preserve"> 10.0 [7.00;14.0]  </t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 17.4 [12.3;23.5]  </t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
         <is>
           <t xml:space="preserve"> &lt;0.001  </t>
         </is>
@@ -679,220 +634,190 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Fragil Vig index, Median [25th;75th]</t>
+          <t>Commorbidity and complexity, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0.36 [0.28;0.48]</t>
+          <t>20.2 [15.0;25.9]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.36 [0.28;0.44]</t>
+          <t>18.3 [13.4;23.4]</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.36 [0.24;0.48]</t>
+          <t>18.1 [13.7;22.8]</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.36 [0.24;0.52]</t>
+          <t xml:space="preserve"> 17.1 [12.2;23.3]  </t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.40 [0.28;0.48]  </t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.491  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PCC, N (%)</t>
+          <t>Fragil Vig index, Median [25th;75th]</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1526 (78.3%)  </t>
+          <t>0.36 [0.28;0.44]</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  591 (83.5%)   </t>
+          <t>0.34 [0.24;0.45]</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  151 (54.3%)   </t>
+          <t>0.36 [0.24;0.48]</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  274 (80.8%)   </t>
+          <t xml:space="preserve"> 0.36 [0.28;0.48]  </t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">    510 (81.7%)    </t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.246  </t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MACA, N (%)</t>
+          <t>PCC, N (%)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  160 (8.21%)   </t>
+          <t xml:space="preserve">  619 (79.3%)   </t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   63 (8.90%)   </t>
+          <t xml:space="preserve">  165 (52.9%)   </t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   31 (11.2%)   </t>
+          <t xml:space="preserve">  317 (77.1%)   </t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   27 (7.96%)   </t>
+          <t xml:space="preserve">    562 (78.1%)    </t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    39 (6.25%)     </t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.077  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dependency according to Barthel Index for Activities of Daily Living, N (%):</t>
+          <t>MACA, N (%)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   77 (9.86%)   </t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   31 (9.94%)   </t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   32 (7.79%)   </t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    46 (6.39%)     </t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.008  </t>
+          <t xml:space="preserve">  0.068  </t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Total (&lt;20)</t>
+          <t>Dependency according to Barthel Index for Activities of Daily Living, N (%):</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  208 (10.7%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   67 (9.46%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   28 (10.1%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   38 (11.2%)   </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">    75 (12.0%)     </t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Severe (20-35)</t>
+          <t xml:space="preserve">    Total (&lt;20)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  256 (13.1%)   </t>
+          <t xml:space="preserve">   69 (8.83%)   </t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   84 (11.9%)   </t>
+          <t xml:space="preserve">   30 (9.62%)   </t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   41 (14.7%)   </t>
+          <t xml:space="preserve">   40 (9.73%)   </t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   45 (13.3%)   </t>
+          <t xml:space="preserve">    77 (10.7%)     </t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    86 (13.8%)     </t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -901,35 +826,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Moderate (40-55)</t>
+          <t xml:space="preserve">    Severe (20-35)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  453 (23.2%)   </t>
+          <t xml:space="preserve">   87 (11.1%)   </t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  140 (19.8%)   </t>
+          <t xml:space="preserve">   40 (12.8%)   </t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   72 (25.9%)   </t>
+          <t xml:space="preserve">   47 (11.4%)   </t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   71 (20.9%)   </t>
+          <t xml:space="preserve">    95 (13.2%)     </t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    170 (27.2%)    </t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -938,35 +858,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Low (60-99)</t>
+          <t xml:space="preserve">    Moderate (40-55)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  991 (50.8%)   </t>
+          <t xml:space="preserve">  148 (19.0%)   </t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  407 (57.5%)   </t>
+          <t xml:space="preserve">   77 (24.7%)   </t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  130 (46.8%)   </t>
+          <t xml:space="preserve">   83 (20.2%)   </t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  175 (51.6%)   </t>
+          <t xml:space="preserve">    187 (26.0%)    </t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    279 (44.7%)    </t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -975,35 +890,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    None (100)</t>
+          <t xml:space="preserve">    Low (60-99)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   33 (1.69%)   </t>
+          <t xml:space="preserve">  463 (59.3%)   </t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (1.13%)    </t>
+          <t xml:space="preserve">  156 (50.0%)   </t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   5 (1.80%)    </t>
+          <t xml:space="preserve">  205 (49.9%)   </t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   7 (2.06%)    </t>
+          <t xml:space="preserve">    320 (44.4%)    </t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    13 (2.08%)     </t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1012,35 +922,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    None (100)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (0.41%)    </t>
+          <t xml:space="preserve">   11 (1.41%)   </t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2 (0.28%)    </t>
+          <t xml:space="preserve">   7 (2.24%)    </t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2 (0.72%)    </t>
+          <t xml:space="preserve">   11 (2.68%)   </t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.88%)    </t>
+          <t xml:space="preserve">    17 (2.36%)     </t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     1 (0.16%)     </t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1049,109 +954,94 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Braden, N (%):</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   3 (0.38%)    </t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   2 (0.64%)    </t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   25 (6.08%)   </t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    24 (3.33%)     </t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Very high (≤9 to 12)</t>
+          <t>Braden, N (%):</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   88 (4.52%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   30 (4.24%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   7 (2.52%)    </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   20 (5.90%)   </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">    31 (4.97%)     </t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Moderate (13-14)</t>
+          <t xml:space="preserve">    Very high (≤9 to 12)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  192 (9.85%)   </t>
+          <t xml:space="preserve">   31 (3.97%)   </t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   52 (7.34%)   </t>
+          <t xml:space="preserve">   6 (1.92%)    </t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   26 (9.35%)   </t>
+          <t xml:space="preserve">   23 (5.60%)   </t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   52 (15.3%)   </t>
+          <t xml:space="preserve">    33 (4.58%)     </t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    62 (9.94%)     </t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1160,35 +1050,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    None or Low (15 to 18)</t>
+          <t xml:space="preserve">    Moderate (13-14)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1632 (83.7%)  </t>
+          <t xml:space="preserve">   50 (6.40%)   </t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  617 (87.1%)   </t>
+          <t xml:space="preserve">   29 (9.29%)   </t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  233 (83.8%)   </t>
+          <t xml:space="preserve">   57 (13.9%)   </t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  256 (75.5%)   </t>
+          <t xml:space="preserve">    68 (9.44%)     </t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    526 (84.3%)    </t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1197,35 +1082,30 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    None or Low (15 to 18)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   37 (1.90%)   </t>
+          <t xml:space="preserve">  678 (86.8%)   </t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   9 (1.27%)    </t>
+          <t xml:space="preserve">  267 (85.6%)   </t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   12 (4.32%)   </t>
+          <t xml:space="preserve">  289 (70.3%)   </t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   11 (3.24%)   </t>
+          <t xml:space="preserve">    583 (81.0%)    </t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     5 (0.80%)     </t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1234,109 +1114,94 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Short Portable Mental Status Questionnaire, N (%):</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   22 (2.82%)   </t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   10 (3.21%)   </t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   42 (10.2%)   </t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    36 (5.00%)     </t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.182  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    No deficit (0-2 mistakes)</t>
+          <t>Short Portable Mental Status Questionnaire, N (%):</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1060 (54.4%)  </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  387 (54.7%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  147 (52.9%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  191 (56.3%)   </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    335 (53.7%)    </t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Low (3-4 mistakes)</t>
+          <t xml:space="preserve">    No deficit (0-2 mistakes)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  288 (14.8%)   </t>
+          <t xml:space="preserve">  432 (55.3%)   </t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  110 (15.5%)   </t>
+          <t xml:space="preserve">  177 (56.7%)   </t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">   39 (14.0%)   </t>
+          <t xml:space="preserve">  227 (55.2%)   </t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">   48 (14.2%)   </t>
+          <t xml:space="preserve">    383 (53.2%)    </t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    91 (14.6%)     </t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1345,35 +1210,30 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Moderate (5-7 mistakes)</t>
+          <t xml:space="preserve">    Low (3-4 mistakes)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  266 (13.6%)   </t>
+          <t xml:space="preserve">  119 (15.2%)   </t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   79 (11.2%)   </t>
+          <t xml:space="preserve">   42 (13.5%)   </t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   42 (15.1%)   </t>
+          <t xml:space="preserve">   53 (12.9%)   </t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   47 (13.9%)   </t>
+          <t xml:space="preserve">    101 (14.0%)    </t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    98 (15.7%)     </t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1382,35 +1242,30 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Severe (8-10 mistakes)</t>
+          <t xml:space="preserve">    Moderate (5-7 mistakes)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  322 (16.5%)   </t>
+          <t xml:space="preserve">   88 (11.3%)   </t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  129 (18.2%)   </t>
+          <t xml:space="preserve">   44 (14.1%)   </t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   45 (16.2%)   </t>
+          <t xml:space="preserve">   52 (12.7%)   </t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   50 (14.7%)   </t>
+          <t xml:space="preserve">    99 (13.8%)     </t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    98 (15.7%)     </t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1419,35 +1274,30 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    Severe (8-10 mistakes)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   13 (0.67%)   </t>
+          <t xml:space="preserve">  136 (17.4%)   </t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.42%)    </t>
+          <t xml:space="preserve">   45 (14.4%)   </t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   5 (1.80%)    </t>
+          <t xml:space="preserve">   55 (13.4%)   </t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.88%)    </t>
+          <t xml:space="preserve">    108 (15.0%)    </t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     2 (0.32%)     </t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1456,109 +1306,94 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Incontinence, N (%):</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   6 (0.77%)    </t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   4 (1.28%)    </t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   24 (5.84%)   </t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    29 (4.03%)     </t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.051  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Fecal and urinary</t>
+          <t>Incontinence, N (%):</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  248 (12.7%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">   91 (12.9%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">   44 (15.8%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">   46 (13.6%)   </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">    67 (10.7%)     </t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve">  0.079  </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Fecal</t>
+          <t xml:space="preserve">    Fecal and urinary</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (0.41%)    </t>
+          <t xml:space="preserve">   87 (11.1%)   </t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">   5 (0.71%)    </t>
+          <t xml:space="preserve">   42 (13.5%)   </t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2 (0.72%)    </t>
+          <t xml:space="preserve">   45 (10.9%)   </t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1 (0.29%)    </t>
+          <t xml:space="preserve">    67 (9.31%)     </t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1567,35 +1402,30 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Urinary</t>
+          <t xml:space="preserve">    Fecal</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1002 (51.4%)  </t>
+          <t xml:space="preserve">   5 (0.64%)    </t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  374 (52.8%)   </t>
+          <t xml:space="preserve">   2 (0.64%)    </t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  150 (54.0%)   </t>
+          <t xml:space="preserve">   1 (0.24%)    </t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">  165 (48.7%)   </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    313 (50.2%)    </t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1604,35 +1434,30 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    None/None registered</t>
+          <t xml:space="preserve">    Urinary</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  691 (35.5%)   </t>
+          <t xml:space="preserve">  352 (45.1%)   </t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  238 (33.6%)   </t>
+          <t xml:space="preserve">  145 (46.5%)   </t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   82 (29.5%)   </t>
+          <t xml:space="preserve">  166 (40.4%)   </t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">  127 (37.5%)   </t>
+          <t xml:space="preserve">    312 (43.3%)    </t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    244 (39.1%)    </t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1641,109 +1466,94 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Social risk, N (%):</t>
+          <t xml:space="preserve">    None/None registered</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  337 (43.1%)   </t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  123 (39.4%)   </t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  199 (48.4%)   </t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    341 (47.4%)    </t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    No</t>
+          <t>Social risk, N (%):</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1165 (59.8%)  </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  558 (78.8%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  177 (63.7%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  149 (44.0%)   </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    281 (45.0%)    </t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Yes</t>
+          <t xml:space="preserve">    No</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  231 (11.9%)   </t>
+          <t xml:space="preserve">  617 (79.0%)   </t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">   71 (10.0%)   </t>
+          <t xml:space="preserve">  193 (61.9%)   </t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">   93 (33.5%)   </t>
+          <t xml:space="preserve">  168 (40.9%)   </t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">   18 (5.31%)   </t>
+          <t xml:space="preserve">    315 (43.8%)    </t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    49 (7.85%)     </t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1752,35 +1562,30 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    Yes</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  553 (28.4%)   </t>
+          <t xml:space="preserve">   74 (9.48%)   </t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   79 (11.2%)   </t>
+          <t xml:space="preserve">  109 (34.9%)   </t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (2.88%)    </t>
+          <t xml:space="preserve">   18 (4.38%)   </t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  172 (50.7%)   </t>
+          <t xml:space="preserve">    50 (6.94%)     </t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    294 (47.1%)    </t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1789,109 +1594,94 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Social Risk (TIRS categorized), N (%):</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   90 (11.5%)   </t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   10 (3.21%)   </t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  225 (54.7%)   </t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    355 (49.3%)    </t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">    no</t>
+          <t>Social Risk (TIRS categorized), N (%):</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1321 (67.8%)  </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  420 (59.3%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  206 (74.1%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  235 (69.3%)   </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">    460 (73.7%)    </t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">    si</t>
+          <t xml:space="preserve">    no</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  618 (31.7%)   </t>
+          <t xml:space="preserve">  454 (58.1%)   </t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  286 (40.4%)   </t>
+          <t xml:space="preserve">  222 (71.2%)   </t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">   71 (25.5%)   </t>
+          <t xml:space="preserve">  263 (64.0%)   </t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  101 (29.8%)   </t>
+          <t xml:space="preserve">    508 (70.6%)    </t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    160 (25.6%)    </t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1900,35 +1690,30 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    'Missing'</t>
+          <t xml:space="preserve">    si</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   10 (0.51%)   </t>
+          <t xml:space="preserve">  323 (41.4%)   </t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2 (0.28%)    </t>
+          <t xml:space="preserve">   89 (28.5%)   </t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1 (0.36%)    </t>
+          <t xml:space="preserve">  115 (28.0%)   </t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.88%)    </t>
+          <t xml:space="preserve">    178 (24.7%)    </t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     4 (0.64%)     </t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -1937,72 +1722,62 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Social Risk (TIRS numeric), Median [25th;75th]</t>
+          <t xml:space="preserve">    'Missing'</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">   4 (0.51%)    </t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">   1 (0.32%)    </t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">   33 (8.03%)   </t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>0.00 [0.00;1.00]</t>
+          <t xml:space="preserve">    34 (4.72%)     </t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 0.00 [0.00;1.00]  </t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Living alone, N (%)</t>
+          <t>Social Risk (TIRS numeric), Median [25th;75th]</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  383 (19.7%)   </t>
+          <t>0.00 [0.00;1.00]</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  182 (25.7%)   </t>
+          <t>0.00 [0.00;1.00]</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   59 (21.2%)   </t>
+          <t>0.00 [0.00;1.00]</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   38 (11.2%)   </t>
+          <t xml:space="preserve"> 0.00 [0.00;1.00]  </t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    104 (16.7%)    </t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
         <is>
           <t xml:space="preserve"> &lt;0.001  </t>
         </is>
@@ -2011,35 +1786,30 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Need for any household adaptation, N (%)</t>
+          <t>Living alone, N (%)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  510 (26.2%)   </t>
+          <t xml:space="preserve">  197 (25.2%)   </t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  246 (34.7%)   </t>
+          <t xml:space="preserve">   71 (22.8%)   </t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   66 (23.7%)   </t>
+          <t xml:space="preserve">   45 (10.9%)   </t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   68 (20.1%)   </t>
+          <t xml:space="preserve">    115 (16.0%)    </t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    130 (20.8%)    </t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
         <is>
           <t xml:space="preserve"> &lt;0.001  </t>
         </is>
@@ -2048,86 +1818,76 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Healthcare center, N (%):</t>
+          <t>Need for any household adaptation, N (%)</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">  284 (36.4%)   </t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   87 (27.9%)   </t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   77 (18.7%)   </t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    141 (19.6%)    </t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.000  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Equip_Atdom</t>
+          <t>Healthcare center, N (%):</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  708 (36.3%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   708 (100%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve">  0.000  </t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Equip_Inf</t>
+          <t xml:space="preserve">    Equip_Atdom</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">  278 (14.3%)   </t>
+          <t xml:space="preserve">   781 (100%)   </t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2137,20 +1897,15 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   278 (100%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2159,35 +1914,30 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">    UAB_consulta</t>
+          <t xml:space="preserve">    Equip_Inf</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">  963 (49.4%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
+          <t xml:space="preserve">   312 (100%)   </t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
           <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">   339 (100%)   </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    624 (100%)     </t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2196,86 +1946,76 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>organit_atdom_2, N (%):</t>
+          <t xml:space="preserve">    UAB_consulta</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">   411 (100%)   </t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">                </t>
+          <t xml:space="preserve">    720 (100%)     </t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   </t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.000  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Borrell</t>
+          <t>organit_atdom_2, N (%):</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">  394 (20.2%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">  394 (55.6%)   </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">                </t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">                   </t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">         </t>
+          <t xml:space="preserve">  0.000  </t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Casanova</t>
+          <t xml:space="preserve">    Borrell</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  278 (14.3%)   </t>
+          <t xml:space="preserve">  440 (56.3%)   </t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2285,20 +2025,15 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">   278 (100%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2307,35 +2042,30 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Montnegre_1</t>
+          <t xml:space="preserve">    Casanova</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">  183 (9.39%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
+          <t xml:space="preserve">   312 (100%)   </t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
           <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
-        </is>
-      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">  183 (54.0%)   </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2344,12 +2074,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Montnegre_2</t>
+          <t xml:space="preserve">    Montnegre_1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  156 (8.00%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2359,20 +2089,15 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">  224 (54.5%)   </t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  156 (46.0%)   </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2381,12 +2106,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Marc_Aureli</t>
+          <t xml:space="preserve">    Montnegre_2</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  287 (14.7%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2396,20 +2121,15 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">  187 (45.5%)   </t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    287 (46.0%)    </t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2418,12 +2138,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Sant_Elies</t>
+          <t xml:space="preserve">    Marc_Aureli</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  337 (17.3%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2438,15 +2158,10 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">    330 (45.8%)    </t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    337 (54.0%)    </t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2455,17 +2170,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Lluch</t>
+          <t xml:space="preserve">    Sant_Elies</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  314 (16.1%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  314 (44.4%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2475,15 +2190,10 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0 (0.00%)    </t>
+          <t xml:space="preserve">    390 (54.2%)    </t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     0 (0.00%)     </t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
         <is>
           <t xml:space="preserve">         </t>
         </is>
@@ -2492,703 +2202,640 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Heart failure, N (%)</t>
+          <t xml:space="preserve">    Lluch</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">  475 (24.4%)   </t>
+          <t xml:space="preserve">  341 (43.7%)   </t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">  212 (29.9%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">   60 (21.6%)   </t>
+          <t xml:space="preserve">   0 (0.00%)    </t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">   79 (23.3%)   </t>
+          <t xml:space="preserve">     0 (0.00%)     </t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">    124 (19.9%)    </t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">         </t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Ischemic heart disease, N (%)</t>
+          <t>Heart failure, N (%)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">  239 (12.3%)   </t>
+          <t xml:space="preserve">  201 (25.7%)   </t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">   81 (11.4%)   </t>
+          <t xml:space="preserve">   57 (18.3%)   </t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">   37 (13.3%)   </t>
+          <t xml:space="preserve">   77 (18.7%)   </t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">   39 (11.5%)   </t>
+          <t xml:space="preserve">    127 (17.6%)    </t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">    82 (13.1%)     </t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.716  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Arrhythmias, N (%)</t>
+          <t>Ischemic heart disease, N (%)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  646 (33.1%)   </t>
+          <t xml:space="preserve">   80 (10.2%)   </t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  237 (33.5%)   </t>
+          <t xml:space="preserve">   36 (11.5%)   </t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  101 (36.3%)   </t>
+          <t xml:space="preserve">   37 (9.00%)   </t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  108 (31.9%)   </t>
+          <t xml:space="preserve">    80 (11.1%)     </t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">    200 (32.1%)    </t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.594  </t>
+          <t xml:space="preserve">  0.641  </t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Dementia, N (%)</t>
+          <t>Arrhythmias, N (%)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">  413 (21.2%)   </t>
+          <t xml:space="preserve">  225 (28.8%)   </t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">  166 (23.4%)   </t>
+          <t xml:space="preserve">   96 (30.8%)   </t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   58 (20.9%)   </t>
+          <t xml:space="preserve">  106 (25.8%)   </t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   72 (21.2%)   </t>
+          <t xml:space="preserve">    198 (27.5%)    </t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">    117 (18.8%)    </t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.221  </t>
+          <t xml:space="preserve">  0.474  </t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Parkinson, N (%)</t>
+          <t>Dementia, N (%)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">  164 (8.41%)   </t>
+          <t xml:space="preserve">  152 (19.5%)   </t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">   56 (7.91%)   </t>
+          <t xml:space="preserve">   54 (17.3%)   </t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">   11 (3.96%)   </t>
+          <t xml:space="preserve">   71 (17.3%)   </t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">   27 (7.96%)   </t>
+          <t xml:space="preserve">    117 (16.2%)    </t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">    70 (11.2%)     </t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.003  </t>
+          <t xml:space="preserve">  0.426  </t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Stroke, N (%)</t>
+          <t>Parkinson, N (%)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">  366 (18.8%)   </t>
+          <t xml:space="preserve">   52 (6.66%)   </t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">  136 (19.2%)   </t>
+          <t xml:space="preserve">   11 (3.53%)   </t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   47 (16.9%)   </t>
+          <t xml:space="preserve">   26 (6.33%)   </t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   71 (20.9%)   </t>
+          <t xml:space="preserve">    68 (9.44%)     </t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">    112 (17.9%)    </t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.562  </t>
+          <t xml:space="preserve">  0.005  </t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Diabetes, N (%)</t>
+          <t>Stroke, N (%)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">  468 (24.0%)   </t>
+          <t xml:space="preserve">  129 (16.5%)   </t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">  207 (29.2%)   </t>
+          <t xml:space="preserve">   43 (13.8%)   </t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">   60 (21.6%)   </t>
+          <t xml:space="preserve">   71 (17.3%)   </t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">   82 (24.2%)   </t>
+          <t xml:space="preserve">    109 (15.1%)    </t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">    119 (19.1%)    </t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.540  </t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Hyperlipidemia, N (%)</t>
+          <t>Diabetes, N (%)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">  287 (14.7%)   </t>
+          <t xml:space="preserve">  193 (24.7%)   </t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">  163 (23.0%)   </t>
+          <t xml:space="preserve">   59 (18.9%)   </t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">   41 (14.7%)   </t>
+          <t xml:space="preserve">   80 (19.5%)   </t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">   31 (9.14%)   </t>
+          <t xml:space="preserve">    118 (16.4%)    </t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">    52 (8.33%)     </t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.001  </t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Chronic Kidney Disease, N (%)</t>
+          <t>Hyperlipidemia, N (%)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  691 (35.5%)   </t>
+          <t xml:space="preserve">  151 (19.3%)   </t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  252 (35.6%)   </t>
+          <t xml:space="preserve">   39 (12.5%)   </t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">   92 (33.1%)   </t>
+          <t xml:space="preserve">   31 (7.54%)   </t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  133 (39.2%)   </t>
+          <t xml:space="preserve">    50 (6.94%)     </t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">    214 (34.3%)    </t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.367  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>COPD, N (%)</t>
+          <t>Chronic Kidney Disease, N (%)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">  357 (18.3%)   </t>
+          <t xml:space="preserve">  236 (30.2%)   </t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">  134 (18.9%)   </t>
+          <t xml:space="preserve">   86 (27.6%)   </t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">   46 (16.5%)   </t>
+          <t xml:space="preserve">  131 (31.9%)   </t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">   67 (19.8%)   </t>
+          <t xml:space="preserve">    211 (29.3%)    </t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">    110 (17.6%)    </t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.698  </t>
+          <t xml:space="preserve">  0.629  </t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Respiratory failure, N (%)</t>
+          <t>COPD, N (%)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   55 (2.82%)   </t>
+          <t xml:space="preserve">  129 (16.5%)   </t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   17 (2.40%)   </t>
+          <t xml:space="preserve">   45 (14.4%)   </t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1 (0.36%)    </t>
+          <t xml:space="preserve">   67 (16.3%)   </t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   8 (2.36%)    </t>
+          <t xml:space="preserve">    110 (15.3%)    </t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">    29 (4.65%)     </t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.002  </t>
+          <t xml:space="preserve">  0.808  </t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Osteoarthritis, N (%)</t>
+          <t>Respiratory failure, N (%)</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1095 (56.2%)  </t>
+          <t xml:space="preserve">   14 (1.79%)   </t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">  389 (54.9%)   </t>
+          <t xml:space="preserve">   1 (0.32%)    </t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">  179 (64.4%)   </t>
+          <t xml:space="preserve">   8 (1.95%)    </t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">  193 (56.9%)   </t>
+          <t xml:space="preserve">    31 (4.31%)     </t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">    334 (53.5%)    </t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.019  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Hip fracture, N (%)</t>
+          <t>Osteoarthritis, N (%)</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">   23 (1.18%)   </t>
+          <t xml:space="preserve">  369 (47.2%)   </t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">   10 (1.41%)   </t>
+          <t xml:space="preserve">  169 (54.2%)   </t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2 (0.72%)    </t>
+          <t xml:space="preserve">  190 (46.2%)   </t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3 (0.88%)    </t>
+          <t xml:space="preserve">    329 (45.7%)    </t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t xml:space="preserve">     8 (1.28%)     </t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.800  </t>
+          <t xml:space="preserve">  0.079  </t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Osteoporosis, N (%)</t>
+          <t>Hip fracture, N (%)</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  536 (27.5%)   </t>
+          <t xml:space="preserve">   8 (1.02%)    </t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  215 (30.4%)   </t>
+          <t xml:space="preserve">   2 (0.64%)    </t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">  107 (38.5%)   </t>
+          <t xml:space="preserve">   3 (0.73%)    </t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">   72 (21.2%)   </t>
+          <t xml:space="preserve">     8 (1.11%)     </t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t xml:space="preserve">    142 (22.8%)    </t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.854  </t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Depression, N (%)</t>
+          <t>Osteoporosis, N (%)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">  578 (29.7%)   </t>
+          <t xml:space="preserve">  200 (25.6%)   </t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">  231 (32.6%)   </t>
+          <t xml:space="preserve">  104 (33.3%)   </t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">   87 (31.3%)   </t>
+          <t xml:space="preserve">   72 (17.5%)   </t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">   91 (26.8%)   </t>
+          <t xml:space="preserve">    141 (19.6%)    </t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">    169 (27.1%)    </t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.085  </t>
+          <t xml:space="preserve"> &lt;0.001  </t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Anxiety, N (%)</t>
+          <t>Depression, N (%)</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">  540 (27.7%)   </t>
+          <t xml:space="preserve">  215 (27.5%)   </t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">  187 (26.4%)   </t>
+          <t xml:space="preserve">   83 (26.6%)   </t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">   94 (33.8%)   </t>
+          <t xml:space="preserve">   91 (22.1%)   </t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">   74 (21.8%)   </t>
+          <t xml:space="preserve">    166 (23.1%)    </t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t xml:space="preserve">    185 (29.6%)    </t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.005  </t>
+          <t xml:space="preserve">  0.096  </t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Anemia, N (%)</t>
+          <t>Anxiety, N (%)</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">  230 (11.8%)   </t>
+          <t xml:space="preserve">  176 (22.5%)   </t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">   91 (12.9%)   </t>
+          <t xml:space="preserve">   89 (28.5%)   </t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">   28 (10.1%)   </t>
+          <t xml:space="preserve">   74 (18.0%)   </t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">   35 (10.3%)   </t>
+          <t xml:space="preserve">    184 (25.6%)    </t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">    76 (12.2%)     </t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.503  </t>
+          <t xml:space="preserve">  0.004  </t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Urinary tract infection, N (%)</t>
+          <t>Anemia, N (%)</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">  448 (23.0%)   </t>
+          <t xml:space="preserve">   81 (10.4%)   </t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">  215 (30.4%)   </t>
+          <t xml:space="preserve">   26 (8.33%)   </t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">   63 (22.7%)   </t>
+          <t xml:space="preserve">   34 (8.27%)   </t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">   72 (21.2%)   </t>
+          <t xml:space="preserve">    78 (10.8%)     </t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t xml:space="preserve">    98 (15.7%)     </t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> &lt;0.001  </t>
+          <t xml:space="preserve">  0.394  </t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>Urinary tract infection, N (%)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  205 (26.2%)   </t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   59 (18.9%)   </t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   71 (17.3%)   </t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    96 (13.3%)     </t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> &lt;0.001  </t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
           <t>Glaucoma, N (%)</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  312 (16.0%)   </t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  113 (16.0%)   </t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   59 (21.2%)   </t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   45 (13.3%)   </t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    95 (15.2%)     </t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  0.050  </t>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  106 (13.6%)   </t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   56 (17.9%)   </t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   45 (10.9%)   </t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    94 (13.1%)     </t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  0.053  </t>
         </is>
       </c>
     </row>

</xml_diff>